<commit_message>
remove the raw pcn values larger than 25 for fitting
</commit_message>
<xml_diff>
--- a/data/biology_results/PCN RNAp results.xlsx
+++ b/data/biology_results/PCN RNAp results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/igem/Documents/copy-number/data/biology_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA42E231-4779-4F46-ACF1-3B3378C04EB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EBE6168-7FB4-3341-9CAC-B6BC71460FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="19420" windowHeight="10300" xr2:uid="{3B59D030-0E93-D54B-8E0B-1AE9133AA16A}"/>
+    <workbookView xWindow="1180" yWindow="940" windowWidth="22420" windowHeight="13300" xr2:uid="{3B59D030-0E93-D54B-8E0B-1AE9133AA16A}"/>
   </bookViews>
   <sheets>
     <sheet name="ddPCR - RNAp" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
update ranp fit to use only selected measurements for fitting
</commit_message>
<xml_diff>
--- a/data/biology_results/PCN RNAp results.xlsx
+++ b/data/biology_results/PCN RNAp results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/igem/Documents/copy-number/data/biology_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EBE6168-7FB4-3341-9CAC-B6BC71460FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DB7269-374A-2644-BB95-2292896BB5DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1180" yWindow="940" windowWidth="22420" windowHeight="13300" xr2:uid="{3B59D030-0E93-D54B-8E0B-1AE9133AA16A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="ddPCR - RNAp" sheetId="1" r:id="rId1"/>
     <sheet name="Our qPCR - RNAp" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,6 +28,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="61">
   <si>
     <t>ddpcr</t>
   </si>
@@ -742,6 +743,9 @@
   </si>
   <si>
     <t>is in the article</t>
+  </si>
+  <si>
+    <t>use for fit</t>
   </si>
 </sst>
 </file>
@@ -1162,7 +1166,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC112E6-EB44-D74A-9EBB-173D582D515E}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
@@ -1171,7 +1175,7 @@
     <col min="4" max="4" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -1190,8 +1194,11 @@
       <c r="F1" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1210,8 +1217,11 @@
       <c r="F2" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1230,8 +1240,11 @@
       <c r="F3" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -1250,8 +1263,11 @@
       <c r="F4" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1270,8 +1286,11 @@
       <c r="F5" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -1290,8 +1309,11 @@
       <c r="F6" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1310,8 +1332,11 @@
       <c r="F7" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1330,8 +1355,11 @@
       <c r="F8" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -1350,8 +1378,11 @@
       <c r="F9" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1370,8 +1401,11 @@
       <c r="F10" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>10</v>
       </c>
@@ -1390,8 +1424,11 @@
       <c r="F11" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -1410,8 +1447,11 @@
       <c r="F12" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
@@ -1428,6 +1468,9 @@
         <v>16</v>
       </c>
       <c r="F13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1439,7 +1482,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AF70DD-E277-4518-9E0E-F1B922B2FC62}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -1448,7 +1491,7 @@
     <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>41</v>
       </c>
@@ -1461,8 +1504,11 @@
       <c r="D1" s="3" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>32</v>
       </c>
@@ -1475,8 +1521,11 @@
       <c r="D2" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
@@ -1489,8 +1538,11 @@
       <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>34</v>
       </c>
@@ -1503,8 +1555,11 @@
       <c r="D4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
@@ -1517,8 +1572,11 @@
       <c r="D5" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>36</v>
       </c>
@@ -1531,8 +1589,11 @@
       <c r="D6" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E6" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
@@ -1545,8 +1606,11 @@
       <c r="D7" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
@@ -1559,8 +1623,11 @@
       <c r="D8" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>39</v>
       </c>
@@ -1573,8 +1640,11 @@
       <c r="D9" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>40</v>
       </c>
@@ -1587,8 +1657,11 @@
       <c r="D10" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E10" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
@@ -1601,8 +1674,11 @@
       <c r="D11" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E11" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>45</v>
       </c>
@@ -1615,8 +1691,11 @@
       <c r="D12" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E12" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>47</v>
       </c>
@@ -1629,8 +1708,11 @@
       <c r="D13" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E13" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>49</v>
       </c>
@@ -1643,8 +1725,11 @@
       <c r="D14" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E14" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>

</xml_diff>

<commit_message>
remove sequences with mutations out of rnap promoter, and update sequences for fit
</commit_message>
<xml_diff>
--- a/data/biology_results/PCN RNAp results.xlsx
+++ b/data/biology_results/PCN RNAp results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/igem/Documents/copy-number/data/biology_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DB7269-374A-2644-BB95-2292896BB5DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31A274E-0B23-CE40-945C-629D5ED36EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="940" windowWidth="22420" windowHeight="13300" xr2:uid="{3B59D030-0E93-D54B-8E0B-1AE9133AA16A}"/>
+    <workbookView xWindow="1980" yWindow="-17200" windowWidth="22420" windowHeight="13300" activeTab="1" xr2:uid="{3B59D030-0E93-D54B-8E0B-1AE9133AA16A}"/>
   </bookViews>
   <sheets>
     <sheet name="ddPCR - RNAp" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="59">
   <si>
     <t>ddpcr</t>
   </si>
@@ -680,12 +680,6 @@
   </si>
   <si>
     <t>mut7</t>
-  </si>
-  <si>
-    <t>mut8</t>
-  </si>
-  <si>
-    <t>mut9</t>
   </si>
   <si>
     <t>Variant name</t>
@@ -832,7 +826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -850,6 +844,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1195,7 +1192,7 @@
         <v>30</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1310,7 +1307,7 @@
         <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -1379,7 +1376,7 @@
         <v>17</v>
       </c>
       <c r="G9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -1402,7 +1399,7 @@
         <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1425,7 +1422,7 @@
         <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1471,7 +1468,7 @@
         <v>17</v>
       </c>
       <c r="G13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1482,7 +1479,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AF70DD-E277-4518-9E0E-F1B922B2FC62}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -1491,29 +1488,29 @@
     <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C2" s="1">
         <v>11.103424110837977</v>
@@ -1524,13 +1521,14 @@
       <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C3" s="1">
         <v>164.36922398734828</v>
@@ -1541,13 +1539,14 @@
       <c r="E3" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C4" s="1">
         <v>56.799580374415605</v>
@@ -1556,15 +1555,16 @@
         <v>17</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C5" s="1">
         <v>188.73429878309068</v>
@@ -1575,13 +1575,14 @@
       <c r="E5" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C6" s="4">
         <v>120.1436013787656</v>
@@ -1592,13 +1593,14 @@
       <c r="E6" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C7" s="1">
         <v>68.830682196579616</v>
@@ -1607,15 +1609,16 @@
         <v>17</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C8" s="1">
         <v>197.97114992640601</v>
@@ -1626,50 +1629,53 @@
       <c r="E8" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C9" s="1">
-        <v>232.00478424258966</v>
+        <v>177.7060168236651</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="C10" s="1">
-        <v>174.6858083205164</v>
+        <v>167.47507574461812</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>43</v>
+        <v>16</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C11" s="1">
-        <v>177.7060168236651</v>
+        <v>153.27099067267383</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>16</v>
@@ -1677,16 +1683,17 @@
       <c r="E11" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C12" s="1">
-        <v>167.47507574461812</v>
+        <v>144.29032164612678</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>16</v>
@@ -1694,45 +1701,13 @@
       <c r="E12" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="1">
-        <v>153.27099067267383</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="1">
-        <v>144.29032164612678</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="F13" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>